<commit_message>
Sync with revised manuscript: ED2 panel labels in figure scripts, droplet morphometry counts (387 droplets/342 beads, two 2-bead droplets), SD3 TOST margin cell fix (87.0), README updates (new title, 27 scripts, ED1-6/SD1-6 mapping)
</commit_message>
<xml_diff>
--- a/Supplementary_Data_3.xlsx
+++ b/Supplementary_Data_3.xlsx
@@ -1759,6 +1759,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -1826,6 +1827,7 @@
         <v>11</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -1840,7 +1842,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-32.74403048033128</v>
+        <v>87.00539999999999</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -2129,8 +2131,6 @@
           <t>Bayes factor</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>B_12 = 0.8670 (inconclusive)</t>
@@ -2153,7 +2153,6 @@
           <t>0.995377</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2241,7 +2240,6 @@
           <t>2698</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2392,8 +2390,6 @@
           <t>kappa=0.5802, beta=3708, b=4.15e-05</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2411,7 +2407,6 @@
           <t>4PL fit = 0.9992; R2 limit = 0.9951</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2429,7 +2424,6 @@
           <t>4PL B = 1.014</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">

</xml_diff>